<commit_message>
delete (Teran et al., 2019) from VEGF:VEGFR2
</commit_message>
<xml_diff>
--- a/data/binding_affinity.xlsx
+++ b/data/binding_affinity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yunjeong/Documents/repos/meta-analysis-for-VEGF-signaling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01A05304-86C4-A440-8D0B-FC577D95D2EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB1F4A2-4A85-634B-8F1E-2F0B3A7844E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22400" yWindow="500" windowWidth="22400" windowHeight="22900" activeTab="1" xr2:uid="{A8742877-6D88-CF4E-82A9-6C281EC17BAE}"/>
   </bookViews>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="34">
   <si>
     <t>Reference</t>
   </si>
@@ -1253,16 +1253,16 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="1">
+      <c r="B9" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="20">
         <v>9.8000000000000007</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="21">
         <v>0.4</v>
       </c>
       <c r="G9" t="s">
@@ -1278,18 +1278,18 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="20" t="s">
+    <row r="10" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="20">
+      <c r="B10" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="8">
         <f>AVERAGE(I12:I14)</f>
         <v>580</v>
       </c>
-      <c r="D10" s="21">
+      <c r="D10" s="9">
         <f>STDEVA(I12:I14)/SQRT(3)</f>
         <v>156.31165450257808</v>
       </c>
@@ -1306,19 +1306,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="8">
-        <v>8600</v>
-      </c>
-      <c r="D11" s="9">
-        <v>500</v>
-      </c>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="G11" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
change value for `Ito & Claesson-Welsh, 1999` from 91.54 pM to 54 pM in VEGF:VEGFR1 sheet
</commit_message>
<xml_diff>
--- a/data/binding_affinity.xlsx
+++ b/data/binding_affinity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yunjeong/Documents/repos/meta-analysis-for-VEGF-signaling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB1F4A2-4A85-634B-8F1E-2F0B3A7844E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{578363E1-483B-6F45-BFC3-7360BABFA36E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22400" yWindow="500" windowWidth="22400" windowHeight="22900" activeTab="1" xr2:uid="{A8742877-6D88-CF4E-82A9-6C281EC17BAE}"/>
+    <workbookView xWindow="22400" yWindow="500" windowWidth="22400" windowHeight="22900" xr2:uid="{A8742877-6D88-CF4E-82A9-6C281EC17BAE}"/>
   </bookViews>
   <sheets>
     <sheet name="VEGFA165_VEGFR1" sheetId="3" r:id="rId1"/>
@@ -1025,7 +1025,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="8">
-        <v>91.54</v>
+        <v>54</v>
       </c>
       <c r="D9" s="9"/>
     </row>

</xml_diff>

<commit_message>
delete (Teran et al., 2019) from VEGF:VEGFR1 sheet
</commit_message>
<xml_diff>
--- a/data/binding_affinity.xlsx
+++ b/data/binding_affinity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yunjeong/Documents/repos/meta-analysis-for-VEGF-signaling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{578363E1-483B-6F45-BFC3-7360BABFA36E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B2C3A54-C8EE-1A4A-A46B-06BA0C39BEFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22400" yWindow="500" windowWidth="22400" windowHeight="22900" xr2:uid="{A8742877-6D88-CF4E-82A9-6C281EC17BAE}"/>
   </bookViews>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="33">
   <si>
     <t>Reference</t>
   </si>
@@ -235,9 +235,6 @@
   </si>
   <si>
     <t>Unpublished data</t>
-  </si>
-  <si>
-    <t>Teran et al., 2019</t>
   </si>
   <si>
     <t>Breier et al., 1995</t>
@@ -902,7 +899,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC68B970-3B91-2544-A9A4-014D1F0CD0C8}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
@@ -925,7 +922,7 @@
     </row>
     <row r="2" spans="1:4" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B2" s="16" t="s">
         <v>8</v>
@@ -996,38 +993,24 @@
         <v>26</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="20">
-        <v>196</v>
-      </c>
-      <c r="D7" s="21">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="D7" s="21"/>
+    </row>
+    <row r="8" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="20">
-        <v>114</v>
-      </c>
-      <c r="D8" s="21"/>
-    </row>
-    <row r="9" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="8">
+      <c r="C8" s="8">
         <v>54</v>
       </c>
-      <c r="D9" s="9"/>
+      <c r="D8" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1128,7 +1111,7 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>8</v>
@@ -1178,7 +1161,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>8</v>
@@ -1395,7 +1378,7 @@
         <v>0.82</v>
       </c>
       <c r="F2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G2">
         <v>5.29</v>
@@ -1403,7 +1386,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>8</v>
@@ -1458,7 +1441,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" s="20" t="s">
         <v>8</v>

</xml_diff>